<commit_message>
# .MC -> EUR
</commit_message>
<xml_diff>
--- a/14_stocks_analysis/01_rankings_sector/2604_cyclical.xlsx
+++ b/14_stocks_analysis/01_rankings_sector/2604_cyclical.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ebc00a0f969ad489/Programmazione/github/FromZeroToQuant-/14_stocks_analysis/01_rankings_sector/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{382F6B64-EE1A-49A6-8695-82CA3B04504A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AF62AA8-80AB-41B2-9052-06F4D4D197B5}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{382F6B64-EE1A-49A6-8695-82CA3B04504A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C01D899-F69D-4599-ADC3-2B88BA085CDA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{865F5E0C-FDB0-40DD-AA47-87F283C01697}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="312">
   <si>
     <t>Symbol</t>
   </si>
@@ -80,51 +80,30 @@
     <t>6.0</t>
   </si>
   <si>
-    <t>3.0</t>
-  </si>
-  <si>
     <t>9.0</t>
   </si>
   <si>
     <t>1.63</t>
   </si>
   <si>
-    <t>-2.65</t>
-  </si>
-  <si>
     <t>4.0</t>
   </si>
   <si>
-    <t>-2.48</t>
-  </si>
-  <si>
     <t>-2.42</t>
   </si>
   <si>
     <t>-2.25</t>
   </si>
   <si>
-    <t>2.10</t>
-  </si>
-  <si>
     <t>-2.81</t>
   </si>
   <si>
-    <t>21.51B</t>
-  </si>
-  <si>
     <t>Bloomin' Brands, Inc.</t>
   </si>
   <si>
     <t>BLMN</t>
   </si>
   <si>
-    <t>518.53M</t>
-  </si>
-  <si>
-    <t>+146.84</t>
-  </si>
-  <si>
     <t>-23.29</t>
   </si>
   <si>
@@ -134,48 +113,12 @@
     <t>RICK</t>
   </si>
   <si>
-    <t>221.16M</t>
-  </si>
-  <si>
-    <t>+108.67</t>
-  </si>
-  <si>
-    <t>1.77</t>
-  </si>
-  <si>
-    <t>-2.51</t>
-  </si>
-  <si>
-    <t>Crown Holdings, Inc.</t>
-  </si>
-  <si>
-    <t>CCK</t>
-  </si>
-  <si>
-    <t>11.20B</t>
-  </si>
-  <si>
-    <t>+85.48</t>
-  </si>
-  <si>
-    <t>2.29</t>
-  </si>
-  <si>
-    <t>-4.02</t>
-  </si>
-  <si>
     <t>Frontdoor, Inc.</t>
   </si>
   <si>
     <t>FTDR</t>
   </si>
   <si>
-    <t>4.85B</t>
-  </si>
-  <si>
-    <t>+22.01</t>
-  </si>
-  <si>
     <t>3.53</t>
   </si>
   <si>
@@ -188,12 +131,6 @@
     <t>WING</t>
   </si>
   <si>
-    <t>4.48B</t>
-  </si>
-  <si>
-    <t>+96.77</t>
-  </si>
-  <si>
     <t>2.32</t>
   </si>
   <si>
@@ -206,15 +143,6 @@
     <t>AMS.MC</t>
   </si>
   <si>
-    <t>25.34B</t>
-  </si>
-  <si>
-    <t>+53.65</t>
-  </si>
-  <si>
-    <t>3.52</t>
-  </si>
-  <si>
     <t>-3.11</t>
   </si>
   <si>
@@ -224,12 +152,6 @@
     <t>ARKO</t>
   </si>
   <si>
-    <t>748.99M</t>
-  </si>
-  <si>
-    <t>+80.94</t>
-  </si>
-  <si>
     <t>2.49</t>
   </si>
   <si>
@@ -242,12 +164,6 @@
     <t>FLXS</t>
   </si>
   <si>
-    <t>304.36M</t>
-  </si>
-  <si>
-    <t>+61.23</t>
-  </si>
-  <si>
     <t>5.00</t>
   </si>
   <si>
@@ -257,81 +173,30 @@
     <t>PET.TO</t>
   </si>
   <si>
-    <t>1.07B</t>
-  </si>
-  <si>
-    <t>+62.00</t>
-  </si>
-  <si>
     <t>2.70</t>
   </si>
   <si>
     <t>-2.56</t>
   </si>
   <si>
-    <t>Chow Tai Fook Jewellery Group Limited</t>
-  </si>
-  <si>
-    <t>1929.HK</t>
-  </si>
-  <si>
-    <t>13.55B</t>
-  </si>
-  <si>
-    <t>+50.14</t>
-  </si>
-  <si>
-    <t>3.38</t>
-  </si>
-  <si>
-    <t>-2.52</t>
-  </si>
-  <si>
     <t>Vistry Group PLC</t>
   </si>
   <si>
     <t>VTY.L</t>
   </si>
   <si>
-    <t>1.47B</t>
-  </si>
-  <si>
-    <t>+106.14</t>
-  </si>
-  <si>
     <t>2.15</t>
   </si>
   <si>
     <t>-2.01</t>
   </si>
   <si>
-    <t>adidas AG</t>
-  </si>
-  <si>
-    <t>ADS.DE</t>
-  </si>
-  <si>
-    <t>31.00B</t>
-  </si>
-  <si>
-    <t>+104.98</t>
-  </si>
-  <si>
-    <t>3.19</t>
-  </si>
-  <si>
     <t>Cars.com Inc.</t>
   </si>
   <si>
     <t>CARS</t>
   </si>
   <si>
-    <t>667.06M</t>
-  </si>
-  <si>
-    <t>+56.01</t>
-  </si>
-  <si>
     <t>0.49</t>
   </si>
   <si>
@@ -344,12 +209,6 @@
     <t>BZH</t>
   </si>
   <si>
-    <t>578.56M</t>
-  </si>
-  <si>
-    <t>+40.00</t>
-  </si>
-  <si>
     <t>1.71</t>
   </si>
   <si>
@@ -362,12 +221,6 @@
     <t>DECK</t>
   </si>
   <si>
-    <t>15.02B</t>
-  </si>
-  <si>
-    <t>+39.07</t>
-  </si>
-  <si>
     <t>9.90</t>
   </si>
   <si>
@@ -380,12 +233,6 @@
     <t>4012.SR</t>
   </si>
   <si>
-    <t>387.66M</t>
-  </si>
-  <si>
-    <t>+37.37</t>
-  </si>
-  <si>
     <t>7.98</t>
   </si>
   <si>
@@ -398,12 +245,6 @@
     <t>CMG</t>
   </si>
   <si>
-    <t>43.70B</t>
-  </si>
-  <si>
-    <t>+35.62</t>
-  </si>
-  <si>
     <t>5.99</t>
   </si>
   <si>
@@ -416,45 +257,18 @@
     <t>TSCO</t>
   </si>
   <si>
-    <t>18.00B</t>
-  </si>
-  <si>
-    <t>+36.18</t>
-  </si>
-  <si>
     <t>4.34</t>
   </si>
   <si>
     <t>-3.21</t>
   </si>
   <si>
-    <t>Harley-Davidson, Inc.</t>
-  </si>
-  <si>
-    <t>HOG</t>
-  </si>
-  <si>
-    <t>2.94B</t>
-  </si>
-  <si>
-    <t>+35.10</t>
-  </si>
-  <si>
-    <t>-5.38</t>
-  </si>
-  <si>
     <t>Red Rock Resorts, Inc.</t>
   </si>
   <si>
     <t>RRR</t>
   </si>
   <si>
-    <t>3.13B</t>
-  </si>
-  <si>
-    <t>+118.32</t>
-  </si>
-  <si>
     <t>1.57</t>
   </si>
   <si>
@@ -467,30 +281,12 @@
     <t>LCII</t>
   </si>
   <si>
-    <t>2.91B</t>
-  </si>
-  <si>
-    <t>+36.00</t>
-  </si>
-  <si>
-    <t>3.48</t>
-  </si>
-  <si>
-    <t>-2.85</t>
-  </si>
-  <si>
     <t>Ferrari N.V.</t>
   </si>
   <si>
     <t>RACE.MI</t>
   </si>
   <si>
-    <t>61.50B</t>
-  </si>
-  <si>
-    <t>+27.11</t>
-  </si>
-  <si>
     <t>6.58</t>
   </si>
   <si>
@@ -503,12 +299,6 @@
     <t>TRIP</t>
   </si>
   <si>
-    <t>1.42B</t>
-  </si>
-  <si>
-    <t>+46.42</t>
-  </si>
-  <si>
     <t>1.67</t>
   </si>
   <si>
@@ -518,177 +308,51 @@
     <t>YETI</t>
   </si>
   <si>
-    <t>3.24B</t>
-  </si>
-  <si>
-    <t>+28.56</t>
-  </si>
-  <si>
     <t>6.56</t>
   </si>
   <si>
     <t>-3.05</t>
   </si>
   <si>
-    <t>Alamar Foods Company</t>
-  </si>
-  <si>
-    <t>6014.SR</t>
-  </si>
-  <si>
-    <t>308.71M</t>
-  </si>
-  <si>
-    <t>+32.47</t>
-  </si>
-  <si>
-    <t>3.49</t>
-  </si>
-  <si>
-    <t>-2.39</t>
-  </si>
-  <si>
     <t>Expedia Group, Inc.</t>
   </si>
   <si>
     <t>EXPE</t>
   </si>
   <si>
-    <t>31.37B</t>
-  </si>
-  <si>
-    <t>+24.40</t>
-  </si>
-  <si>
     <t>1.72</t>
   </si>
   <si>
-    <t>Aristocrat Leisure Limited</t>
-  </si>
-  <si>
-    <t>ALL.AX</t>
-  </si>
-  <si>
-    <t>+23.27</t>
-  </si>
-  <si>
-    <t>9.14</t>
-  </si>
-  <si>
-    <t>-2.37</t>
-  </si>
-  <si>
     <t>Winpak Ltd.</t>
   </si>
   <si>
     <t>WPK.TO</t>
   </si>
   <si>
-    <t>1.75B</t>
-  </si>
-  <si>
-    <t>+22.72</t>
-  </si>
-  <si>
     <t>10.82</t>
   </si>
   <si>
     <t>-2.34</t>
   </si>
   <si>
-    <t>BANDAI NAMCO Holdings Inc.</t>
-  </si>
-  <si>
-    <t>7832.T</t>
-  </si>
-  <si>
-    <t>14.91B</t>
-  </si>
-  <si>
-    <t>+20.13</t>
-  </si>
-  <si>
-    <t>8.14</t>
-  </si>
-  <si>
     <t>Richelieu Hardware Ltd.</t>
   </si>
   <si>
     <t>RCH.TO</t>
   </si>
   <si>
-    <t>1.59B</t>
-  </si>
-  <si>
-    <t>+13.28</t>
-  </si>
-  <si>
     <t>5.97</t>
   </si>
   <si>
     <t>-5.77</t>
   </si>
   <si>
-    <t>Build-A-Bear Workshop, Inc.</t>
-  </si>
-  <si>
-    <t>BBW</t>
-  </si>
-  <si>
-    <t>476.03M</t>
-  </si>
-  <si>
-    <t>+15.95</t>
-  </si>
-  <si>
-    <t>5.23</t>
-  </si>
-  <si>
-    <t>-3.02</t>
-  </si>
-  <si>
-    <t>HASEKO Corporation</t>
-  </si>
-  <si>
-    <t>1808.T</t>
-  </si>
-  <si>
-    <t>4.66B</t>
-  </si>
-  <si>
-    <t>+13.33</t>
-  </si>
-  <si>
-    <t>2.85</t>
-  </si>
-  <si>
-    <t>Marriott International, Inc.</t>
-  </si>
-  <si>
-    <t>MAR</t>
-  </si>
-  <si>
-    <t>97.44B</t>
-  </si>
-  <si>
-    <t>+11.59</t>
-  </si>
-  <si>
-    <t>3.77</t>
-  </si>
-  <si>
     <t>Macy's, Inc.</t>
   </si>
   <si>
     <t>M</t>
   </si>
   <si>
-    <t>5.31B</t>
-  </si>
-  <si>
-    <t>+207.87</t>
-  </si>
-  <si>
     <t>2.06</t>
   </si>
   <si>
@@ -701,78 +365,30 @@
     <t>3092.T</t>
   </si>
   <si>
-    <t>5.79B</t>
-  </si>
-  <si>
-    <t>+150.77</t>
-  </si>
-  <si>
-    <t>10.77</t>
-  </si>
-  <si>
-    <t>-2.23</t>
-  </si>
-  <si>
     <t>DENSO Corporation</t>
   </si>
   <si>
     <t>6902.T</t>
   </si>
   <si>
-    <t>32.57B</t>
-  </si>
-  <si>
-    <t>+48.59</t>
-  </si>
-  <si>
-    <t>3.02</t>
-  </si>
-  <si>
     <t>Churchill Downs Incorporated</t>
   </si>
   <si>
     <t>CHDN</t>
   </si>
   <si>
-    <t>6.94B</t>
-  </si>
-  <si>
-    <t>+47.92</t>
-  </si>
-  <si>
     <t>1.44</t>
   </si>
   <si>
     <t>-3.17</t>
   </si>
   <si>
-    <t>Shenzhou International Group Holdings Limited</t>
-  </si>
-  <si>
-    <t>2313.HK</t>
-  </si>
-  <si>
-    <t>8.98B</t>
-  </si>
-  <si>
-    <t>+44.10</t>
-  </si>
-  <si>
-    <t>4.19</t>
-  </si>
-  <si>
     <t>Autoliv, Inc.</t>
   </si>
   <si>
     <t>ALV</t>
   </si>
   <si>
-    <t>8.67B</t>
-  </si>
-  <si>
-    <t>+28.59</t>
-  </si>
-  <si>
     <t>2.96</t>
   </si>
   <si>
@@ -785,12 +401,6 @@
     <t>WGO</t>
   </si>
   <si>
-    <t>904.94M</t>
-  </si>
-  <si>
-    <t>+43.88</t>
-  </si>
-  <si>
     <t>2.58</t>
   </si>
   <si>
@@ -803,12 +413,6 @@
     <t>SBH</t>
   </si>
   <si>
-    <t>1.39B</t>
-  </si>
-  <si>
-    <t>+32.82</t>
-  </si>
-  <si>
     <t>2.38</t>
   </si>
   <si>
@@ -821,30 +425,12 @@
     <t>BYD</t>
   </si>
   <si>
-    <t>6.60B</t>
-  </si>
-  <si>
-    <t>+28.14</t>
-  </si>
-  <si>
-    <t>2.46</t>
-  </si>
-  <si>
-    <t>-4.00</t>
-  </si>
-  <si>
     <t>Lear Corporation</t>
   </si>
   <si>
     <t>LEA</t>
   </si>
   <si>
-    <t>6.55B</t>
-  </si>
-  <si>
-    <t>+19.95</t>
-  </si>
-  <si>
     <t>6.05</t>
   </si>
   <si>
@@ -857,12 +443,6 @@
     <t>SCVL</t>
   </si>
   <si>
-    <t>510.56M</t>
-  </si>
-  <si>
-    <t>+24.67</t>
-  </si>
-  <si>
     <t>3.13</t>
   </si>
   <si>
@@ -875,97 +455,523 @@
     <t>LOCO</t>
   </si>
   <si>
-    <t>396.61M</t>
-  </si>
-  <si>
-    <t>+21.65</t>
-  </si>
-  <si>
     <t>-3.34</t>
   </si>
   <si>
-    <t>Adient plc</t>
-  </si>
-  <si>
-    <t>ADNT</t>
-  </si>
-  <si>
-    <t>1.67B</t>
-  </si>
-  <si>
-    <t>+20.93</t>
-  </si>
-  <si>
-    <t>-3.41</t>
-  </si>
-  <si>
-    <t>Nathan's Famous, Inc.</t>
-  </si>
-  <si>
-    <t>NATH</t>
-  </si>
-  <si>
-    <t>409.82M</t>
-  </si>
-  <si>
-    <t>+16.54</t>
-  </si>
-  <si>
-    <t>9.50</t>
-  </si>
-  <si>
-    <t>Monarch Casino &amp; Resort, Inc.</t>
-  </si>
-  <si>
-    <t>MCRI</t>
-  </si>
-  <si>
-    <t>2.12B</t>
-  </si>
-  <si>
-    <t>+2.76</t>
-  </si>
-  <si>
-    <t>8.42</t>
-  </si>
-  <si>
-    <t>-3.13</t>
-  </si>
-  <si>
-    <t>United Parks &amp; Resorts Inc.</t>
-  </si>
-  <si>
-    <t>PRKS</t>
-  </si>
-  <si>
-    <t>1.94B</t>
-  </si>
-  <si>
-    <t>+59.11</t>
-  </si>
-  <si>
-    <t>1.87</t>
-  </si>
-  <si>
-    <t>0.32</t>
-  </si>
-  <si>
-    <t>Albany International Corp.</t>
-  </si>
-  <si>
-    <t>AIN</t>
-  </si>
-  <si>
-    <t>1.63B</t>
-  </si>
-  <si>
-    <t>+30.94</t>
-  </si>
-  <si>
-    <t>2.66</t>
-  </si>
-  <si>
-    <t>-2.45</t>
+    <t>489.55M</t>
+  </si>
+  <si>
+    <t>+161.44</t>
+  </si>
+  <si>
+    <t>3.04B</t>
+  </si>
+  <si>
+    <t>+124.38</t>
+  </si>
+  <si>
+    <t>758.62M</t>
+  </si>
+  <si>
+    <t>+78.64</t>
+  </si>
+  <si>
+    <t>302.70M</t>
+  </si>
+  <si>
+    <t>+62.11</t>
+  </si>
+  <si>
+    <t>4.09B</t>
+  </si>
+  <si>
+    <t>+115.52</t>
+  </si>
+  <si>
+    <t>1.05B</t>
+  </si>
+  <si>
+    <t>+65.86</t>
+  </si>
+  <si>
+    <t>5.20B</t>
+  </si>
+  <si>
+    <t>+214.60</t>
+  </si>
+  <si>
+    <t>5.76B</t>
+  </si>
+  <si>
+    <t>+105.60</t>
+  </si>
+  <si>
+    <t>9.81</t>
+  </si>
+  <si>
+    <t>-2.80</t>
+  </si>
+  <si>
+    <t>6.47B</t>
+  </si>
+  <si>
+    <t>+58.55</t>
+  </si>
+  <si>
+    <t>676.70M</t>
+  </si>
+  <si>
+    <t>+53.78</t>
+  </si>
+  <si>
+    <t>536.90M</t>
+  </si>
+  <si>
+    <t>+50.86</t>
+  </si>
+  <si>
+    <t>6.70B</t>
+  </si>
+  <si>
+    <t>+17.28</t>
+  </si>
+  <si>
+    <t>Group 1 Automotive, Inc.</t>
+  </si>
+  <si>
+    <t>GPI</t>
+  </si>
+  <si>
+    <t>4.12B</t>
+  </si>
+  <si>
+    <t>+46.37</t>
+  </si>
+  <si>
+    <t>-23.50</t>
+  </si>
+  <si>
+    <t>-3.63</t>
+  </si>
+  <si>
+    <t>4.58B</t>
+  </si>
+  <si>
+    <t>+29.03</t>
+  </si>
+  <si>
+    <t>The Berkeley Group Holdings plc</t>
+  </si>
+  <si>
+    <t>BKG.L</t>
+  </si>
+  <si>
+    <t>4.28B</t>
+  </si>
+  <si>
+    <t>+80.95</t>
+  </si>
+  <si>
+    <t>3.46</t>
+  </si>
+  <si>
+    <t>-2.47</t>
+  </si>
+  <si>
+    <t>Shatirah House Restaurant Co.</t>
+  </si>
+  <si>
+    <t>6016.SR</t>
+  </si>
+  <si>
+    <t>116.29M</t>
+  </si>
+  <si>
+    <t>+43.69</t>
+  </si>
+  <si>
+    <t>9.36</t>
+  </si>
+  <si>
+    <t>-3.33</t>
+  </si>
+  <si>
+    <t>Resilient</t>
+  </si>
+  <si>
+    <t>6.44B</t>
+  </si>
+  <si>
+    <t>+39.13</t>
+  </si>
+  <si>
+    <t>2.44</t>
+  </si>
+  <si>
+    <t>-2.96</t>
+  </si>
+  <si>
+    <t>1.36B</t>
+  </si>
+  <si>
+    <t>+35.97</t>
+  </si>
+  <si>
+    <t>BRP Inc.</t>
+  </si>
+  <si>
+    <t>DOO.TO</t>
+  </si>
+  <si>
+    <t>3.93B</t>
+  </si>
+  <si>
+    <t>+26.35</t>
+  </si>
+  <si>
+    <t>2.62</t>
+  </si>
+  <si>
+    <t>-2.75</t>
+  </si>
+  <si>
+    <t>CCL Industries Inc.</t>
+  </si>
+  <si>
+    <t>CCL-B.TO</t>
+  </si>
+  <si>
+    <t>10.72B</t>
+  </si>
+  <si>
+    <t>+17.29</t>
+  </si>
+  <si>
+    <t>4.01</t>
+  </si>
+  <si>
+    <t>-2.62</t>
+  </si>
+  <si>
+    <t>Liquidity Services, Inc.</t>
+  </si>
+  <si>
+    <t>LQDT</t>
+  </si>
+  <si>
+    <t>1.15B</t>
+  </si>
+  <si>
+    <t>-8.52</t>
+  </si>
+  <si>
+    <t>5.66</t>
+  </si>
+  <si>
+    <t>1.45B</t>
+  </si>
+  <si>
+    <t>+107.65</t>
+  </si>
+  <si>
+    <t>Domino's Pizza, Inc.</t>
+  </si>
+  <si>
+    <t>DPZ</t>
+  </si>
+  <si>
+    <t>11.22B</t>
+  </si>
+  <si>
+    <t>+47.49</t>
+  </si>
+  <si>
+    <t>3.01</t>
+  </si>
+  <si>
+    <t>-2.41</t>
+  </si>
+  <si>
+    <t>Sonoco Products Company</t>
+  </si>
+  <si>
+    <t>SON</t>
+  </si>
+  <si>
+    <t>5.02B</t>
+  </si>
+  <si>
+    <t>+77.67</t>
+  </si>
+  <si>
+    <t>1.28</t>
+  </si>
+  <si>
+    <t>-2.30</t>
+  </si>
+  <si>
+    <t>32.74B</t>
+  </si>
+  <si>
+    <t>+44.61</t>
+  </si>
+  <si>
+    <t>3.06</t>
+  </si>
+  <si>
+    <t>14.52B</t>
+  </si>
+  <si>
+    <t>+43.90</t>
+  </si>
+  <si>
+    <t>41.29B</t>
+  </si>
+  <si>
+    <t>+43.53</t>
+  </si>
+  <si>
+    <t>17.12B</t>
+  </si>
+  <si>
+    <t>+43.17</t>
+  </si>
+  <si>
+    <t>25.02B</t>
+  </si>
+  <si>
+    <t>+53.46</t>
+  </si>
+  <si>
+    <t>4.21</t>
+  </si>
+  <si>
+    <t>2.71B</t>
+  </si>
+  <si>
+    <t>+43.08</t>
+  </si>
+  <si>
+    <t>3.17</t>
+  </si>
+  <si>
+    <t>-1.84</t>
+  </si>
+  <si>
+    <t>58.32B</t>
+  </si>
+  <si>
+    <t>+33.39</t>
+  </si>
+  <si>
+    <t>Gentex Corporation</t>
+  </si>
+  <si>
+    <t>GNTX</t>
+  </si>
+  <si>
+    <t>4.86B</t>
+  </si>
+  <si>
+    <t>+42.99</t>
+  </si>
+  <si>
+    <t>0.31</t>
+  </si>
+  <si>
+    <t>-2.46</t>
+  </si>
+  <si>
+    <t>8.73B</t>
+  </si>
+  <si>
+    <t>+27.71</t>
+  </si>
+  <si>
+    <t>223.13M</t>
+  </si>
+  <si>
+    <t>+41.68</t>
+  </si>
+  <si>
+    <t>1.62</t>
+  </si>
+  <si>
+    <t>-2.24</t>
+  </si>
+  <si>
+    <t>Rollins, Inc.</t>
+  </si>
+  <si>
+    <t>ROL</t>
+  </si>
+  <si>
+    <t>26.07B</t>
+  </si>
+  <si>
+    <t>+14.35</t>
+  </si>
+  <si>
+    <t>10.94</t>
+  </si>
+  <si>
+    <t>-2.93</t>
+  </si>
+  <si>
+    <t>Bridgestone Corporation</t>
+  </si>
+  <si>
+    <t>5108.T</t>
+  </si>
+  <si>
+    <t>27.27B</t>
+  </si>
+  <si>
+    <t>+58.96</t>
+  </si>
+  <si>
+    <t>3.54</t>
+  </si>
+  <si>
+    <t>-2.53</t>
+  </si>
+  <si>
+    <t>383.72M</t>
+  </si>
+  <si>
+    <t>+38.48</t>
+  </si>
+  <si>
+    <t>3.15B</t>
+  </si>
+  <si>
+    <t>+32.18</t>
+  </si>
+  <si>
+    <t>482.03M</t>
+  </si>
+  <si>
+    <t>+32.05</t>
+  </si>
+  <si>
+    <t>30.94B</t>
+  </si>
+  <si>
+    <t>+26.13</t>
+  </si>
+  <si>
+    <t>382.57M</t>
+  </si>
+  <si>
+    <t>+26.12</t>
+  </si>
+  <si>
+    <t>1.72B</t>
+  </si>
+  <si>
+    <t>+24.37</t>
+  </si>
+  <si>
+    <t>1.57B</t>
+  </si>
+  <si>
+    <t>+14.51</t>
+  </si>
+  <si>
+    <t>Bath &amp; Body Works, Inc.</t>
+  </si>
+  <si>
+    <t>BBWI</t>
+  </si>
+  <si>
+    <t>3.92B</t>
+  </si>
+  <si>
+    <t>+79.21</t>
+  </si>
+  <si>
+    <t>2.72</t>
+  </si>
+  <si>
+    <t>H&amp;R Block, Inc.</t>
+  </si>
+  <si>
+    <t>HRB</t>
+  </si>
+  <si>
+    <t>3.77B</t>
+  </si>
+  <si>
+    <t>+77.29</t>
+  </si>
+  <si>
+    <t>2.89</t>
+  </si>
+  <si>
+    <t>1.98</t>
+  </si>
+  <si>
+    <t>869.55M</t>
+  </si>
+  <si>
+    <t>+49.73</t>
+  </si>
+  <si>
+    <t>1.41B</t>
+  </si>
+  <si>
+    <t>+46.90</t>
+  </si>
+  <si>
+    <t>KB Home</t>
+  </si>
+  <si>
+    <t>KBH</t>
+  </si>
+  <si>
+    <t>3.05B</t>
+  </si>
+  <si>
+    <t>+28.04</t>
+  </si>
+  <si>
+    <t>3.56</t>
+  </si>
+  <si>
+    <t>-1.28</t>
+  </si>
+  <si>
+    <t>Seera Holding Group</t>
+  </si>
+  <si>
+    <t>1810.SR</t>
+  </si>
+  <si>
+    <t>3.50B</t>
+  </si>
+  <si>
+    <t>+29.27</t>
+  </si>
+  <si>
+    <t>3.09</t>
+  </si>
+  <si>
+    <t>-4.03</t>
+  </si>
+  <si>
+    <t>Asbury Automotive Group, Inc.</t>
+  </si>
+  <si>
+    <t>ABG</t>
+  </si>
+  <si>
+    <t>3.80B</t>
+  </si>
+  <si>
+    <t>+24.20</t>
+  </si>
+  <si>
+    <t>-3.81</t>
   </si>
 </sst>
 </file>
@@ -1385,19 +1391,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>141</v>
       </c>
       <c r="G2" t="s">
         <v>11</v>
@@ -1406,7 +1412,7 @@
         <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="J2" t="s">
         <v>9</v>
@@ -1414,7 +1420,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -1422,28 +1428,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>142</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>143</v>
       </c>
       <c r="G4" t="s">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="H4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J4" t="s">
         <v>9</v>
@@ -1451,7 +1457,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -1465,22 +1471,22 @@
         <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>144</v>
       </c>
       <c r="E6" t="s">
         <v>36</v>
       </c>
       <c r="F6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I6" t="s">
         <v>39</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" t="s">
-        <v>41</v>
       </c>
       <c r="J6" t="s">
         <v>9</v>
@@ -1496,28 +1502,28 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>146</v>
+      </c>
+      <c r="E8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" t="s">
+        <v>147</v>
+      </c>
+      <c r="G8" t="s">
         <v>42</v>
       </c>
-      <c r="C8" t="s">
-        <v>42</v>
-      </c>
-      <c r="D8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" t="s">
-        <v>42</v>
-      </c>
-      <c r="F8" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" t="s">
-        <v>46</v>
-      </c>
       <c r="H8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I8" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="J8" t="s">
         <v>9</v>
@@ -1525,7 +1531,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -1533,28 +1539,28 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>148</v>
       </c>
       <c r="E10" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>149</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="H10" t="s">
         <v>13</v>
       </c>
       <c r="I10" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="J10" t="s">
         <v>9</v>
@@ -1562,7 +1568,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1570,28 +1576,28 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>150</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>57</v>
+        <v>151</v>
       </c>
       <c r="G12" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="H12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I12" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="J12" t="s">
         <v>9</v>
@@ -1599,7 +1605,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -1607,28 +1613,28 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>152</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>103</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>153</v>
       </c>
       <c r="G14" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="H14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I14" t="s">
-        <v>65</v>
+        <v>106</v>
       </c>
       <c r="J14" t="s">
         <v>9</v>
@@ -1636,7 +1642,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>61</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -1644,28 +1650,28 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>154</v>
       </c>
       <c r="E16" t="s">
-        <v>66</v>
+        <v>107</v>
       </c>
       <c r="F16" t="s">
-        <v>69</v>
+        <v>155</v>
       </c>
       <c r="G16" t="s">
-        <v>70</v>
+        <v>156</v>
       </c>
       <c r="H16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I16" t="s">
-        <v>23</v>
+        <v>157</v>
       </c>
       <c r="J16" t="s">
         <v>9</v>
@@ -1673,7 +1679,7 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>67</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -1681,28 +1687,28 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>159</v>
       </c>
       <c r="G18" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="H18" t="s">
         <v>12</v>
       </c>
       <c r="I18" t="s">
-        <v>76</v>
+        <v>114</v>
       </c>
       <c r="J18" t="s">
         <v>9</v>
@@ -1710,7 +1716,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -1718,28 +1724,28 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>160</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="G20" t="s">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="H20" t="s">
         <v>8</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="J20" t="s">
         <v>9</v>
@@ -1747,7 +1753,7 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -1755,28 +1761,28 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="C22" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="D22" t="s">
-        <v>85</v>
+        <v>162</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
       <c r="F22" t="s">
-        <v>86</v>
+        <v>163</v>
       </c>
       <c r="G22" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="H22" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I22" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="J22" t="s">
         <v>9</v>
@@ -1784,7 +1790,7 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -1792,28 +1798,28 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="C24" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>164</v>
       </c>
       <c r="E24" t="s">
-        <v>89</v>
+        <v>129</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
+        <v>165</v>
       </c>
       <c r="G24" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="H24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I24" t="s">
-        <v>82</v>
+        <v>132</v>
       </c>
       <c r="J24" t="s">
         <v>9</v>
@@ -1821,7 +1827,7 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>90</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -1829,28 +1835,28 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
       <c r="D26" t="s">
-        <v>96</v>
+        <v>168</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>166</v>
       </c>
       <c r="F26" t="s">
-        <v>97</v>
+        <v>169</v>
       </c>
       <c r="G26" t="s">
-        <v>98</v>
+        <v>170</v>
       </c>
       <c r="H26" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I26" t="s">
-        <v>99</v>
+        <v>171</v>
       </c>
       <c r="J26" t="s">
         <v>9</v>
@@ -1858,7 +1864,7 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>95</v>
+        <v>167</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -1866,28 +1872,28 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>172</v>
       </c>
       <c r="E28" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="F28" t="s">
-        <v>103</v>
+        <v>173</v>
       </c>
       <c r="G28" t="s">
-        <v>104</v>
+        <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I28" t="s">
-        <v>105</v>
+        <v>28</v>
       </c>
       <c r="J28" t="s">
         <v>9</v>
@@ -1895,7 +1901,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>101</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -1903,28 +1909,28 @@
         <v>15</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>174</v>
       </c>
       <c r="C30" t="s">
-        <v>106</v>
+        <v>174</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>176</v>
       </c>
       <c r="E30" t="s">
-        <v>106</v>
+        <v>174</v>
       </c>
       <c r="F30" t="s">
-        <v>109</v>
+        <v>177</v>
       </c>
       <c r="G30" t="s">
-        <v>110</v>
+        <v>178</v>
       </c>
       <c r="H30" t="s">
         <v>10</v>
       </c>
       <c r="I30" t="s">
-        <v>111</v>
+        <v>179</v>
       </c>
       <c r="J30" t="s">
         <v>9</v>
@@ -1932,7 +1938,7 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>107</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -1940,36 +1946,36 @@
         <v>16</v>
       </c>
       <c r="B32" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="C32" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="D32" t="s">
-        <v>114</v>
+        <v>182</v>
       </c>
       <c r="E32" t="s">
-        <v>112</v>
+        <v>180</v>
       </c>
       <c r="F32" t="s">
-        <v>115</v>
+        <v>183</v>
       </c>
       <c r="G32" t="s">
-        <v>116</v>
+        <v>184</v>
       </c>
       <c r="H32" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I32" t="s">
-        <v>117</v>
+        <v>185</v>
       </c>
       <c r="J32" t="s">
-        <v>9</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>113</v>
+        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -1977,28 +1983,28 @@
         <v>17</v>
       </c>
       <c r="B34" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="C34" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D34" t="s">
-        <v>120</v>
+        <v>187</v>
       </c>
       <c r="E34" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="F34" t="s">
-        <v>121</v>
+        <v>188</v>
       </c>
       <c r="G34" t="s">
-        <v>122</v>
+        <v>189</v>
       </c>
       <c r="H34" t="s">
         <v>13</v>
       </c>
       <c r="I34" t="s">
-        <v>123</v>
+        <v>190</v>
       </c>
       <c r="J34" t="s">
         <v>9</v>
@@ -2006,7 +2012,7 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -2014,28 +2020,28 @@
         <v>18</v>
       </c>
       <c r="B36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D36" t="s">
+        <v>191</v>
+      </c>
+      <c r="E36" t="s">
+        <v>123</v>
+      </c>
+      <c r="F36" t="s">
+        <v>192</v>
+      </c>
+      <c r="G36" t="s">
+        <v>125</v>
+      </c>
+      <c r="H36" t="s">
+        <v>12</v>
+      </c>
+      <c r="I36" t="s">
         <v>126</v>
-      </c>
-      <c r="E36" t="s">
-        <v>124</v>
-      </c>
-      <c r="F36" t="s">
-        <v>127</v>
-      </c>
-      <c r="G36" t="s">
-        <v>128</v>
-      </c>
-      <c r="H36" t="s">
-        <v>10</v>
-      </c>
-      <c r="I36" t="s">
-        <v>129</v>
       </c>
       <c r="J36" t="s">
         <v>9</v>
@@ -2043,7 +2049,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -2051,28 +2057,28 @@
         <v>19</v>
       </c>
       <c r="B38" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="C38" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="D38" t="s">
-        <v>132</v>
+        <v>195</v>
       </c>
       <c r="E38" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="F38" t="s">
-        <v>133</v>
+        <v>196</v>
       </c>
       <c r="G38" t="s">
-        <v>22</v>
+        <v>197</v>
       </c>
       <c r="H38" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I38" t="s">
-        <v>134</v>
+        <v>198</v>
       </c>
       <c r="J38" t="s">
         <v>9</v>
@@ -2080,7 +2086,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>131</v>
+        <v>194</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -2088,28 +2094,28 @@
         <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>135</v>
+        <v>199</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>199</v>
       </c>
       <c r="D40" t="s">
-        <v>137</v>
+        <v>201</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>199</v>
       </c>
       <c r="F40" t="s">
-        <v>138</v>
+        <v>202</v>
       </c>
       <c r="G40" t="s">
-        <v>139</v>
+        <v>203</v>
       </c>
       <c r="H40" t="s">
         <v>12</v>
       </c>
       <c r="I40" t="s">
-        <v>140</v>
+        <v>204</v>
       </c>
       <c r="J40" t="s">
         <v>9</v>
@@ -2117,7 +2123,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>136</v>
+        <v>200</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -2125,28 +2131,28 @@
         <v>21</v>
       </c>
       <c r="B42" t="s">
-        <v>141</v>
+        <v>205</v>
       </c>
       <c r="C42" t="s">
-        <v>141</v>
+        <v>205</v>
       </c>
       <c r="D42" t="s">
-        <v>143</v>
+        <v>207</v>
       </c>
       <c r="E42" t="s">
-        <v>141</v>
+        <v>205</v>
       </c>
       <c r="F42" t="s">
-        <v>144</v>
+        <v>208</v>
       </c>
       <c r="G42" t="s">
-        <v>145</v>
+        <v>209</v>
       </c>
       <c r="H42" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I42" t="s">
-        <v>146</v>
+        <v>17</v>
       </c>
       <c r="J42" t="s">
         <v>9</v>
@@ -2154,7 +2160,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>142</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -2162,28 +2168,28 @@
         <v>22</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>47</v>
       </c>
       <c r="C44" t="s">
-        <v>147</v>
+        <v>47</v>
       </c>
       <c r="D44" t="s">
-        <v>149</v>
+        <v>210</v>
       </c>
       <c r="E44" t="s">
-        <v>147</v>
+        <v>47</v>
       </c>
       <c r="F44" t="s">
-        <v>150</v>
+        <v>211</v>
       </c>
       <c r="G44" t="s">
-        <v>151</v>
+        <v>49</v>
       </c>
       <c r="H44" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I44" t="s">
-        <v>152</v>
+        <v>50</v>
       </c>
       <c r="J44" t="s">
         <v>9</v>
@@ -2191,7 +2197,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>148</v>
+        <v>48</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -2199,28 +2205,28 @@
         <v>23</v>
       </c>
       <c r="B46" t="s">
-        <v>153</v>
+        <v>212</v>
       </c>
       <c r="C46" t="s">
-        <v>153</v>
+        <v>212</v>
       </c>
       <c r="D46" t="s">
-        <v>155</v>
+        <v>214</v>
       </c>
       <c r="E46" t="s">
-        <v>153</v>
+        <v>212</v>
       </c>
       <c r="F46" t="s">
-        <v>156</v>
+        <v>215</v>
       </c>
       <c r="G46" t="s">
-        <v>157</v>
+        <v>216</v>
       </c>
       <c r="H46" t="s">
         <v>12</v>
       </c>
       <c r="I46" t="s">
-        <v>21</v>
+        <v>217</v>
       </c>
       <c r="J46" t="s">
         <v>9</v>
@@ -2228,7 +2234,7 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -2236,28 +2242,28 @@
         <v>24</v>
       </c>
       <c r="B48" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="C48" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="D48" t="s">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="E48" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="F48" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="G48" t="s">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="H48" t="s">
         <v>13</v>
       </c>
       <c r="I48" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="J48" t="s">
         <v>9</v>
@@ -2265,7 +2271,7 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>159</v>
+        <v>219</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
@@ -2273,28 +2279,28 @@
         <v>25</v>
       </c>
       <c r="B50" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="C50" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="D50" t="s">
-        <v>166</v>
+        <v>224</v>
       </c>
       <c r="E50" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="F50" t="s">
-        <v>167</v>
+        <v>225</v>
       </c>
       <c r="G50" t="s">
-        <v>168</v>
+        <v>226</v>
       </c>
       <c r="H50" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I50" t="s">
-        <v>169</v>
+        <v>118</v>
       </c>
       <c r="J50" t="s">
         <v>9</v>
@@ -2302,7 +2308,7 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
-        <v>165</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
@@ -2310,28 +2316,28 @@
         <v>26</v>
       </c>
       <c r="B52" t="s">
-        <v>170</v>
+        <v>59</v>
       </c>
       <c r="C52" t="s">
-        <v>170</v>
+        <v>59</v>
       </c>
       <c r="D52" t="s">
-        <v>172</v>
+        <v>227</v>
       </c>
       <c r="E52" t="s">
-        <v>170</v>
+        <v>59</v>
       </c>
       <c r="F52" t="s">
-        <v>173</v>
+        <v>228</v>
       </c>
       <c r="G52" t="s">
-        <v>174</v>
+        <v>61</v>
       </c>
       <c r="H52" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I52" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="J52" t="s">
         <v>9</v>
@@ -2339,7 +2345,7 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
-        <v>171</v>
+        <v>60</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
@@ -2347,28 +2353,28 @@
         <v>27</v>
       </c>
       <c r="B54" t="s">
-        <v>175</v>
+        <v>67</v>
       </c>
       <c r="C54" t="s">
-        <v>175</v>
+        <v>67</v>
       </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>229</v>
       </c>
       <c r="E54" t="s">
-        <v>175</v>
+        <v>67</v>
       </c>
       <c r="F54" t="s">
-        <v>177</v>
+        <v>230</v>
       </c>
       <c r="G54" t="s">
-        <v>178</v>
+        <v>69</v>
       </c>
       <c r="H54" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I54" t="s">
-        <v>179</v>
+        <v>70</v>
       </c>
       <c r="J54" t="s">
         <v>9</v>
@@ -2376,7 +2382,7 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
-        <v>176</v>
+        <v>68</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
@@ -2384,28 +2390,28 @@
         <v>28</v>
       </c>
       <c r="B56" t="s">
-        <v>180</v>
+        <v>71</v>
       </c>
       <c r="C56" t="s">
-        <v>180</v>
+        <v>71</v>
       </c>
       <c r="D56" t="s">
-        <v>182</v>
+        <v>231</v>
       </c>
       <c r="E56" t="s">
-        <v>180</v>
+        <v>71</v>
       </c>
       <c r="F56" t="s">
-        <v>183</v>
+        <v>232</v>
       </c>
       <c r="G56" t="s">
-        <v>184</v>
+        <v>73</v>
       </c>
       <c r="H56" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I56" t="s">
-        <v>185</v>
+        <v>74</v>
       </c>
       <c r="J56" t="s">
         <v>9</v>
@@ -2413,7 +2419,7 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
-        <v>181</v>
+        <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
@@ -2421,28 +2427,28 @@
         <v>29</v>
       </c>
       <c r="B58" t="s">
-        <v>186</v>
+        <v>33</v>
       </c>
       <c r="C58" t="s">
-        <v>186</v>
+        <v>33</v>
       </c>
       <c r="D58" t="s">
-        <v>188</v>
+        <v>233</v>
       </c>
       <c r="E58" t="s">
-        <v>186</v>
+        <v>33</v>
       </c>
       <c r="F58" t="s">
-        <v>189</v>
+        <v>234</v>
       </c>
       <c r="G58" t="s">
-        <v>190</v>
+        <v>235</v>
       </c>
       <c r="H58" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I58" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="J58" t="s">
         <v>9</v>
@@ -2450,7 +2456,7 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
-        <v>187</v>
+        <v>34</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
@@ -2458,28 +2464,28 @@
         <v>30</v>
       </c>
       <c r="B60" t="s">
-        <v>191</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>191</v>
+        <v>79</v>
       </c>
       <c r="D60" t="s">
-        <v>193</v>
+        <v>236</v>
       </c>
       <c r="E60" t="s">
-        <v>191</v>
+        <v>79</v>
       </c>
       <c r="F60" t="s">
-        <v>194</v>
+        <v>237</v>
       </c>
       <c r="G60" t="s">
-        <v>195</v>
+        <v>238</v>
       </c>
       <c r="H60" t="s">
         <v>8</v>
       </c>
       <c r="I60" t="s">
-        <v>196</v>
+        <v>239</v>
       </c>
       <c r="J60" t="s">
         <v>9</v>
@@ -2487,7 +2493,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
-        <v>192</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
@@ -2495,28 +2501,28 @@
         <v>31</v>
       </c>
       <c r="B62" t="s">
-        <v>197</v>
+        <v>81</v>
       </c>
       <c r="C62" t="s">
-        <v>197</v>
+        <v>81</v>
       </c>
       <c r="D62" t="s">
-        <v>199</v>
+        <v>240</v>
       </c>
       <c r="E62" t="s">
-        <v>197</v>
+        <v>81</v>
       </c>
       <c r="F62" t="s">
-        <v>200</v>
+        <v>241</v>
       </c>
       <c r="G62" t="s">
-        <v>201</v>
+        <v>83</v>
       </c>
       <c r="H62" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I62" t="s">
-        <v>202</v>
+        <v>84</v>
       </c>
       <c r="J62" t="s">
         <v>9</v>
@@ -2524,7 +2530,7 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>198</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
@@ -2532,28 +2538,28 @@
         <v>32</v>
       </c>
       <c r="B64" t="s">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="C64" t="s">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="D64" t="s">
-        <v>205</v>
+        <v>244</v>
       </c>
       <c r="E64" t="s">
-        <v>203</v>
+        <v>242</v>
       </c>
       <c r="F64" t="s">
-        <v>206</v>
+        <v>245</v>
       </c>
       <c r="G64" t="s">
-        <v>207</v>
+        <v>246</v>
       </c>
       <c r="H64" t="s">
         <v>13</v>
       </c>
       <c r="I64" t="s">
-        <v>35</v>
+        <v>247</v>
       </c>
       <c r="J64" t="s">
         <v>9</v>
@@ -2561,7 +2567,7 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>204</v>
+        <v>243</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
@@ -2569,28 +2575,28 @@
         <v>33</v>
       </c>
       <c r="B66" t="s">
-        <v>208</v>
+        <v>115</v>
       </c>
       <c r="C66" t="s">
-        <v>208</v>
+        <v>115</v>
       </c>
       <c r="D66" t="s">
-        <v>210</v>
+        <v>248</v>
       </c>
       <c r="E66" t="s">
-        <v>208</v>
+        <v>115</v>
       </c>
       <c r="F66" t="s">
-        <v>211</v>
+        <v>249</v>
       </c>
       <c r="G66" t="s">
-        <v>212</v>
+        <v>117</v>
       </c>
       <c r="H66" t="s">
         <v>12</v>
       </c>
       <c r="I66" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="J66" t="s">
         <v>9</v>
@@ -2598,7 +2604,7 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>209</v>
+        <v>116</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
@@ -2606,28 +2612,28 @@
         <v>34</v>
       </c>
       <c r="B68" t="s">
-        <v>213</v>
+        <v>23</v>
       </c>
       <c r="C68" t="s">
-        <v>213</v>
+        <v>23</v>
       </c>
       <c r="D68" t="s">
-        <v>215</v>
+        <v>250</v>
       </c>
       <c r="E68" t="s">
-        <v>213</v>
+        <v>23</v>
       </c>
       <c r="F68" t="s">
-        <v>216</v>
+        <v>251</v>
       </c>
       <c r="G68" t="s">
-        <v>217</v>
+        <v>252</v>
       </c>
       <c r="H68" t="s">
         <v>13</v>
       </c>
       <c r="I68" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="J68" t="s">
         <v>9</v>
@@ -2635,7 +2641,7 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
-        <v>214</v>
+        <v>24</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
@@ -2643,28 +2649,28 @@
         <v>35</v>
       </c>
       <c r="B70" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="C70" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="D70" t="s">
-        <v>221</v>
+        <v>256</v>
       </c>
       <c r="E70" t="s">
-        <v>219</v>
+        <v>254</v>
       </c>
       <c r="F70" t="s">
-        <v>222</v>
+        <v>257</v>
       </c>
       <c r="G70" t="s">
-        <v>223</v>
+        <v>258</v>
       </c>
       <c r="H70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I70" t="s">
-        <v>224</v>
+        <v>259</v>
       </c>
       <c r="J70" t="s">
         <v>9</v>
@@ -2672,7 +2678,7 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
-        <v>220</v>
+        <v>255</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
@@ -2680,28 +2686,28 @@
         <v>36</v>
       </c>
       <c r="B72" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="C72" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="D72" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="E72" t="s">
-        <v>225</v>
+        <v>260</v>
       </c>
       <c r="F72" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="G72" t="s">
-        <v>229</v>
+        <v>264</v>
       </c>
       <c r="H72" t="s">
         <v>13</v>
       </c>
       <c r="I72" t="s">
-        <v>20</v>
+        <v>265</v>
       </c>
       <c r="J72" t="s">
         <v>9</v>
@@ -2709,7 +2715,7 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
-        <v>226</v>
+        <v>261</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
@@ -2717,28 +2723,28 @@
         <v>37</v>
       </c>
       <c r="B74" t="s">
-        <v>230</v>
+        <v>63</v>
       </c>
       <c r="C74" t="s">
-        <v>230</v>
+        <v>63</v>
       </c>
       <c r="D74" t="s">
-        <v>232</v>
+        <v>266</v>
       </c>
       <c r="E74" t="s">
-        <v>230</v>
+        <v>63</v>
       </c>
       <c r="F74" t="s">
-        <v>233</v>
+        <v>267</v>
       </c>
       <c r="G74" t="s">
-        <v>234</v>
+        <v>65</v>
       </c>
       <c r="H74" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I74" t="s">
-        <v>235</v>
+        <v>66</v>
       </c>
       <c r="J74" t="s">
         <v>9</v>
@@ -2746,7 +2752,7 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>231</v>
+        <v>64</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
@@ -2754,28 +2760,28 @@
         <v>38</v>
       </c>
       <c r="B76" t="s">
-        <v>236</v>
+        <v>88</v>
       </c>
       <c r="C76" t="s">
-        <v>236</v>
+        <v>88</v>
       </c>
       <c r="D76" t="s">
-        <v>238</v>
+        <v>268</v>
       </c>
       <c r="E76" t="s">
-        <v>236</v>
+        <v>88</v>
       </c>
       <c r="F76" t="s">
-        <v>239</v>
+        <v>269</v>
       </c>
       <c r="G76" t="s">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="H76" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I76" t="s">
-        <v>179</v>
+        <v>91</v>
       </c>
       <c r="J76" t="s">
         <v>9</v>
@@ -2783,7 +2789,7 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>237</v>
+        <v>89</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
@@ -2791,28 +2797,28 @@
         <v>39</v>
       </c>
       <c r="B78" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="C78" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="D78" t="s">
-        <v>243</v>
+        <v>270</v>
       </c>
       <c r="E78" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="F78" t="s">
-        <v>244</v>
+        <v>271</v>
       </c>
       <c r="G78" t="s">
-        <v>245</v>
+        <v>135</v>
       </c>
       <c r="H78" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I78" t="s">
-        <v>246</v>
+        <v>136</v>
       </c>
       <c r="J78" t="s">
         <v>9</v>
@@ -2820,7 +2826,7 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>242</v>
+        <v>134</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
@@ -2828,28 +2834,28 @@
         <v>40</v>
       </c>
       <c r="B80" t="s">
-        <v>247</v>
+        <v>92</v>
       </c>
       <c r="C80" t="s">
-        <v>247</v>
+        <v>92</v>
       </c>
       <c r="D80" t="s">
-        <v>249</v>
+        <v>272</v>
       </c>
       <c r="E80" t="s">
-        <v>247</v>
+        <v>92</v>
       </c>
       <c r="F80" t="s">
-        <v>250</v>
+        <v>273</v>
       </c>
       <c r="G80" t="s">
-        <v>251</v>
+        <v>94</v>
       </c>
       <c r="H80" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I80" t="s">
-        <v>252</v>
+        <v>46</v>
       </c>
       <c r="J80" t="s">
         <v>9</v>
@@ -2857,7 +2863,7 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
-        <v>248</v>
+        <v>93</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
@@ -2865,28 +2871,28 @@
         <v>41</v>
       </c>
       <c r="B82" t="s">
-        <v>253</v>
+        <v>137</v>
       </c>
       <c r="C82" t="s">
-        <v>253</v>
+        <v>137</v>
       </c>
       <c r="D82" t="s">
-        <v>255</v>
+        <v>274</v>
       </c>
       <c r="E82" t="s">
-        <v>253</v>
+        <v>137</v>
       </c>
       <c r="F82" t="s">
-        <v>256</v>
+        <v>275</v>
       </c>
       <c r="G82" t="s">
-        <v>257</v>
+        <v>15</v>
       </c>
       <c r="H82" t="s">
         <v>12</v>
       </c>
       <c r="I82" t="s">
-        <v>258</v>
+        <v>139</v>
       </c>
       <c r="J82" t="s">
         <v>9</v>
@@ -2894,7 +2900,7 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>254</v>
+        <v>138</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
@@ -2902,28 +2908,28 @@
         <v>42</v>
       </c>
       <c r="B84" t="s">
-        <v>259</v>
+        <v>95</v>
       </c>
       <c r="C84" t="s">
-        <v>259</v>
+        <v>95</v>
       </c>
       <c r="D84" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
       <c r="E84" t="s">
-        <v>259</v>
+        <v>95</v>
       </c>
       <c r="F84" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="G84" t="s">
-        <v>263</v>
+        <v>97</v>
       </c>
       <c r="H84" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I84" t="s">
-        <v>264</v>
+        <v>98</v>
       </c>
       <c r="J84" t="s">
         <v>9</v>
@@ -2931,7 +2937,7 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
-        <v>260</v>
+        <v>96</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
@@ -2939,28 +2945,28 @@
         <v>43</v>
       </c>
       <c r="B86" t="s">
-        <v>265</v>
+        <v>99</v>
       </c>
       <c r="C86" t="s">
-        <v>265</v>
+        <v>99</v>
       </c>
       <c r="D86" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="E86" t="s">
-        <v>265</v>
+        <v>99</v>
       </c>
       <c r="F86" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="G86" t="s">
-        <v>269</v>
+        <v>101</v>
       </c>
       <c r="H86" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I86" t="s">
-        <v>270</v>
+        <v>102</v>
       </c>
       <c r="J86" t="s">
         <v>9</v>
@@ -2968,7 +2974,7 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
-        <v>266</v>
+        <v>100</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
@@ -2976,28 +2982,28 @@
         <v>44</v>
       </c>
       <c r="B88" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="C88" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="D88" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="E88" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="F88" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="G88" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
       <c r="H88" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="I88" t="s">
-        <v>276</v>
+        <v>198</v>
       </c>
       <c r="J88" t="s">
         <v>9</v>
@@ -3005,7 +3011,7 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
@@ -3013,28 +3019,28 @@
         <v>45</v>
       </c>
       <c r="B90" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C90" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="D90" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="E90" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="F90" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="G90" t="s">
-        <v>16</v>
+        <v>289</v>
       </c>
       <c r="H90" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I90" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
       <c r="J90" t="s">
         <v>9</v>
@@ -3042,7 +3048,7 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
@@ -3050,28 +3056,28 @@
         <v>46</v>
       </c>
       <c r="B92" t="s">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="C92" t="s">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="D92" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="E92" t="s">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="F92" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="G92" t="s">
-        <v>16</v>
+        <v>121</v>
       </c>
       <c r="H92" t="s">
         <v>10</v>
       </c>
       <c r="I92" t="s">
-        <v>286</v>
+        <v>122</v>
       </c>
       <c r="J92" t="s">
         <v>9</v>
@@ -3079,7 +3085,7 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
-        <v>283</v>
+        <v>120</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
@@ -3087,28 +3093,28 @@
         <v>47</v>
       </c>
       <c r="B94" t="s">
-        <v>287</v>
+        <v>85</v>
       </c>
       <c r="C94" t="s">
-        <v>287</v>
+        <v>85</v>
       </c>
       <c r="D94" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="E94" t="s">
-        <v>287</v>
+        <v>85</v>
       </c>
       <c r="F94" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="G94" t="s">
-        <v>291</v>
+        <v>87</v>
       </c>
       <c r="H94" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="I94" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J94" t="s">
         <v>9</v>
@@ -3116,7 +3122,7 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
-        <v>288</v>
+        <v>86</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
@@ -3124,28 +3130,28 @@
         <v>48</v>
       </c>
       <c r="B96" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C96" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D96" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E96" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F96" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G96" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="H96" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I96" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="J96" t="s">
         <v>9</v>
@@ -3153,7 +3159,7 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
@@ -3161,36 +3167,36 @@
         <v>49</v>
       </c>
       <c r="B98" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C98" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="D98" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E98" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F98" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="G98" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="H98" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I98" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="J98" t="s">
-        <v>9</v>
+        <v>186</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
@@ -3198,28 +3204,28 @@
         <v>50</v>
       </c>
       <c r="B100" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C100" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D100" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="E100" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F100" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="G100" t="s">
-        <v>308</v>
+        <v>11</v>
       </c>
       <c r="H100" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I100" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="J100" t="s">
         <v>9</v>
@@ -3227,7 +3233,7 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>